<commit_message>
trazabilidad de cortes: 11 lecturas de recepcion de Aloha (25-26/09) en calidad_lotes.xlsx (8 lotes + hoja cortes_recepcion) + paneles regenerados
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/calidad_lotes.xlsx
+++ b/fuentes/calidad_lotes.xlsx
@@ -14,11 +14,12 @@
   </bookViews>
   <sheets>
     <sheet name="lotes" sheetId="1" r:id="rId1"/>
+    <sheet name="cortes_recepcion" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">lotes!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'lotes'!$A$1:$Q$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -276,7 +277,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
   <si>
     <t>codigo</t>
   </si>
@@ -360,13 +361,475 @@
   </si>
   <si>
     <t>Corte longitudinal en origen, carga 09/09/2026 (Plan: Cassio programado 09/09, 1008 cajas MIC; semana 37 Cassio 3 camiones a R$ 35, este seria el 2do, Chabat / Maicol). 2 dedos = 4 mitades: pulpa blanco marfil opaca y pareja, sin franja ambar, cascara media bien adherida, seccion redondeada, ovulos alineados, resto floral negro solo en la punta, oxidacion leve normal. Claramente mas verde y pareja que el corte del 08/09 (que tenia 1 de 3 adelantado). Corte 5. Viene con un "informe tecnico de evaluacion de maduracion" en PDF (Von Loesecke grado 1, preclimaterico) que describe lo mismo pero sin fecha, lote, productor ni mediciones: se guarda como referencia, no como dato. Pronostico de ruta al cargar: sin ola de frio si llega el sabado 12; el 13-14/09 Montevideo baja a 5,9 / 4,5 C, no dejarlo cargado el fin de semana. Codigo provisorio: reemplazar por el CK### al recibir.</t>
+  </si>
+  <si>
+    <t>PYAS012</t>
+  </si>
+  <si>
+    <t>Paraguay</t>
+  </si>
+  <si>
+    <t>Paraguay AS</t>
+  </si>
+  <si>
+    <t>maduracion inmediata / venta rapida</t>
+  </si>
+  <si>
+    <t>Pie de camion #268 (Aloha), chofer Celoso Chavez, AAKC666, corte 25/09 07:20. Corte de llegada 2 · Rechazar para guardar: los 5 dedos (frente, medio y fondo) con pulpa amarillo crema pareja y franja ambar en el eje, cascara todavia verde; franja nitida en los dedos 4 y 5 (fondo), dedo 3 (medio) en 3. Maduracion generalizada, no un foco. Sin frio, corona, Moko ni inclusiones. Accion: no va a camara larga; separar el lote, despacho por firmeza; reclamo por maduracion de origen. Camara probable (conteo 26/09): ZAC 4 o 20 (entradas PY del 25/09). Es el camion AS cargado el 21/09 (Aloha: descargado 24/09; el corte se fotografio el 25 a la manana). Lectura IA Opus en Aloha, protocolo UAM v1, confianza MEDIA (tabla gris, sin regla), confirmada por Javier Gonzalez.</t>
+  </si>
+  <si>
+    <t>PYMS021</t>
+  </si>
+  <si>
+    <t>Paraguay MS</t>
+  </si>
+  <si>
+    <t>Pie #270, pallet 30/30, chofer Alfredo Patino, HFZ237, corte 25/09 08:51. Corte 2 · Rechazar para guardar: 5 de 5 con pulpa amarilla de punta a cuello (amarillo manteca), eje ambar nitido, centro translucido en el dedo del medio; cascara verde. El del fondo el menos avanzado, igual virado. Leve pardeo seco en cuello/pedunculo de 3 dedos: CORONA A CONFIRMAR (cortar coronas y puntas aparte). Haces limpios, sin Moko ni frio. Accion: separar el pallet 30/30 y cortar 5 dedos mas de otras posiciones para ver si el camion entero viene asi; reclamo por fruta llegada virando. Camion MS cargado el 21/09 (Aloha: en frontera el 24). Camara probable: ZAC 20 o 6 (PY, entrada 25/09). Confianza MEDIA.</t>
+  </si>
+  <si>
+    <t>SUPREMA-2509</t>
+  </si>
+  <si>
+    <t>Bolivia</t>
+  </si>
+  <si>
+    <t>Banexfrut</t>
+  </si>
+  <si>
+    <t>venta rapida / maduracion inmediata</t>
+  </si>
+  <si>
+    <t>Marca SUPREMA (Banexfrut), pallet 37/40, corte 25/09 10:10. OJO: quedo guardado en el pie #249 (camion del 17/09) pero por marca, fecha del ticket y exportador corresponde al Banexfrut descargado el 25/09 (pie #272, Alex Valverde, 4713IYD, 1050 cajas; cargado el 18/09, 7 dias de viaje). Corte 2 · Rechazar para guardar, con gradiente por posicion: frente y medio amarillos con franja nitida (2), los 2 del fondo crema amarillento con franja leve (3). Buen llenado, cascara verde. Accion: separar, venta rapida; cortar 5 mas de frente y medio para dimensionar cuanta fruta esta en 2. Camara probable: ZAC 30 (750 cajas, sin dia de gas al 26/09) + resto en camara 2 (la foto de la camara 2 decia 423 y el ERP 23: puede ser esta fruta). Confianza MEDIA.</t>
+  </si>
+  <si>
+    <t>PYMS022</t>
+  </si>
+  <si>
+    <t>camara con observacion, rotar primero, prueba de yodo</t>
+  </si>
+  <si>
+    <t>Pie #271, pallet 1/30, chofer Nelson Paez, BBF626, corte 25/09 10:17. OJO: leido con la guia generica de PLATANO, no con el protocolo de banana: su "4 · Marginal" no es un 4 Almar comparable. Describe cascara verde, pulpa crema-amarilla palida, pareja de centro a borde, firme, opaca, sin manchas ni haces marrones; dedos 3 y 4 (centro) algo mas amarillos con la linea de semillas marcada; dedo 5 mas corto y palido. En escala banana: 4 con reserva (3-4). Accion: recibir con observacion, rotar primero; si va a camara, yodo. Camara: ZAC 19 (981 cajas, entrada 25/09 "base 7": coincide exacto con las 981 cajas del camion). Camion MS cargado el 22/09. Confianza MEDIA.</t>
+  </si>
+  <si>
+    <t>FH070</t>
+  </si>
+  <si>
+    <t>Fisher</t>
+  </si>
+  <si>
+    <t>camara corta, prioridad de despacho</t>
+  </si>
+  <si>
+    <t>Pie #273, pallet 3/30, via Etimex, chofer Daniel Ferreira Faria, IZD6D78, corte 25/09 11:08; unica muestra sobre tabla blanca. Corte 3 · Marginal: pulpa crema amarillenta pareja en los 5, franja leve en el eje (dedo 3, medio, el mas adelantado), latex escaso, haces limpios, sin pintas. La IA anoto: "si con la fruta en la mano se ve mas amarilla, baja a 2". Accion: camara corta y prioridad de despacho; cortar 5 mas de la zona del dedo 3. Camion Fischer cargado el 22/09 (Amaro; Aloha: en frontera el 24), 3 dias. Camara probable: ZAC 24 (BR, entradas 24 y 25/09). Confianza MEDIA.</t>
+  </si>
+  <si>
+    <t>BONITA-278</t>
+  </si>
+  <si>
+    <t>Ecuador</t>
+  </si>
+  <si>
+    <t>Noboa (Bonita)</t>
+  </si>
+  <si>
+    <t>camara corta y salida rapida</t>
+  </si>
+  <si>
+    <t>Pie #278, marca BONITA (Noboa), pallet 26/30, placa leida JHF560 (dudosa), chofer Marco Munoz, PYCJ23, corte 26/09 08:27. Corte 3 · Marginal: 4 de 5 en 3 (crema amarillenta, eje apenas virado, franja insinuada, bordes crema), dedo 4 en 4. Punteado y trazos pardos a lo largo del eje en los dedos 1, 2 y 5: lo mas probable ovulos oxidados por el corte, pero con transito largo no se descarta pinta parda por frio subagudo. Accion: si alguna toma de pulpa da menos de 13 C, pelar un dedo de frente y otro de fondo y fotografiar la cara interna de la cascara. Contenedor de Ecuador (no esta en el plan de compras). Confianza MEDIA.</t>
+  </si>
+  <si>
+    <t>PEPE-275</t>
+  </si>
+  <si>
+    <t>Interbanana (Pepe)</t>
+  </si>
+  <si>
+    <t>camara corta o maduracion inmediata; separar el fondo</t>
+  </si>
+  <si>
+    <t>Pie #275, marca PEPE (Interbanana), DOS muestras: pallet 22/30 (08:32) y pallet 25/30 (08:41), chofer Daniel Alvarez, PYCJ24. Muestra 1: 3 · Marginal con 2 de 5 dedos en 2: dedos 1-3 (frente/medio) crema amarillenta con franja leve; dedos 4 y 5 (FONDO) con franja ambar nitida de punta a cuello y brillo humedo (2); dedo 5 delgado con cascara gruesa (llenado corto). Pardeo en cuello de los dedos 1 y 2 (corona, sospecha); restos florales secos en puntas 2, 4 y 5 (vigilar punta de cigarro al madurar). Muestra 2: 3 · Marginal, los 5 en 3, franja leve mas notoria en dedos 4 y 5. El ticket se leyo "carga 05/09, descarga 28/09" (23 dias): seguro mal leido, verificar. Accion: separar la fruta del fondo y cortar 5 mas de esa posicion. Confianza MEDIA.</t>
+  </si>
+  <si>
+    <t>BONITA-279</t>
+  </si>
+  <si>
+    <t>Nobora Trading (Bonita)</t>
+  </si>
+  <si>
+    <t>camara corta con prioridad de despacho (3-4)</t>
+  </si>
+  <si>
+    <t>Pie #279, marca BONITA (Nobora Trading Group), pallet 22/30, placa leida PTC-123, chofer Marcelo Hernandez, VHFH90. DOS lecturas del MISMO pallet: 08:37 = 3 · Marginal (los 5 en 3, franja leve, mas marcada en el del MEDIO; foto mas amarillenta y con peor luz) y 08:46 = 4 · Aceptar (crema pareja y opaca en los 5, sin franja nitida, leve solo en el del medio; secciones redondeadas, haces limpios, cascara verde fina, buen llenado). Tomar como 3-4, no como dos lotes. Accion: camara segun plan; si el gradiente termico supera 4 C, cortar 5 mas del medio; vigilar el medio, que madura primero. Confianza MEDIA.</t>
+  </si>
+  <si>
+    <t>fecha</t>
+  </si>
+  <si>
+    <t>hora</t>
+  </si>
+  <si>
+    <t>pie_camion</t>
+  </si>
+  <si>
+    <t>codigo_lote</t>
+  </si>
+  <si>
+    <t>marca</t>
+  </si>
+  <si>
+    <t>pallet</t>
+  </si>
+  <si>
+    <t>productor_exportador</t>
+  </si>
+  <si>
+    <t>chofer</t>
+  </si>
+  <si>
+    <t>placa</t>
+  </si>
+  <si>
+    <t>dedos_foto</t>
+  </si>
+  <si>
+    <t>puntaje</t>
+  </si>
+  <si>
+    <t>veredicto</t>
+  </si>
+  <si>
+    <t>posicion_adelantada</t>
+  </si>
+  <si>
+    <t>sospechas</t>
+  </si>
+  <si>
+    <t>accion</t>
+  </si>
+  <si>
+    <t>protocolo</t>
+  </si>
+  <si>
+    <t>confianza</t>
+  </si>
+  <si>
+    <t>leido_por</t>
+  </si>
+  <si>
+    <t>confirmado_por</t>
+  </si>
+  <si>
+    <t>nota</t>
+  </si>
+  <si>
+    <t>07:20</t>
+  </si>
+  <si>
+    <t>#268</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Alvaro Saldivar (Paraguay AS)</t>
+  </si>
+  <si>
+    <t>Celoso Chavez</t>
+  </si>
+  <si>
+    <t>AAKC666</t>
+  </si>
+  <si>
+    <t>Rechazar para guardar</t>
+  </si>
+  <si>
+    <t>fondo (dedos 4-5 nitidos); medio en 3</t>
+  </si>
+  <si>
+    <t>ninguna (sin frio, corona, Moko)</t>
+  </si>
+  <si>
+    <t>maduracion inmediata o venta rapida; separar; despacho por firmeza; reclamo maduracion de origen</t>
+  </si>
+  <si>
+    <t>banana UAM v1</t>
+  </si>
+  <si>
+    <t>media</t>
+  </si>
+  <si>
+    <t>IA Opus (Aloha)</t>
+  </si>
+  <si>
+    <t>Javier Gonzalez</t>
+  </si>
+  <si>
+    <t>maduracion generalizada, no un foco</t>
+  </si>
+  <si>
+    <t>08:51</t>
+  </si>
+  <si>
+    <t>#270</t>
+  </si>
+  <si>
+    <t>30/30</t>
+  </si>
+  <si>
+    <t>Milciades Sosa (Paraguay MS)</t>
+  </si>
+  <si>
+    <t>Alfredo Patino</t>
+  </si>
+  <si>
+    <t>HFZ237</t>
+  </si>
+  <si>
+    <t>todos virados; fondo el menos avanzado</t>
+  </si>
+  <si>
+    <t>pardeo seco en cuello/pedunculo de 3 dedos: corona a confirmar</t>
+  </si>
+  <si>
+    <t>maduracion inmediata o venta rapida; separar pallet 30/30; cortar 5 mas de otras posiciones; cortar coronas y puntas; reclamo</t>
+  </si>
+  <si>
+    <t>amarillo manteca punta a cuello, eje ambar nitido, centro translucido en el del medio</t>
+  </si>
+  <si>
+    <t>10:10</t>
+  </si>
+  <si>
+    <t>#272 (guardado en #249)</t>
+  </si>
+  <si>
+    <t>SUPREMA</t>
+  </si>
+  <si>
+    <t>37/40</t>
+  </si>
+  <si>
+    <t>Alex Valverde</t>
+  </si>
+  <si>
+    <t>4713IYD</t>
+  </si>
+  <si>
+    <t>frente y medio (2); fondo en 3</t>
+  </si>
+  <si>
+    <t>ninguna</t>
+  </si>
+  <si>
+    <t>separar; venta rapida o maduracion inmediata; cortar 5 mas de frente y medio</t>
+  </si>
+  <si>
+    <t>guardado en el pie equivocado (#249 del 17/09); corresponde al camion del 25/09</t>
+  </si>
+  <si>
+    <t>10:17</t>
+  </si>
+  <si>
+    <t>#271</t>
+  </si>
+  <si>
+    <t>1/30</t>
+  </si>
+  <si>
+    <t>Nelson Paez</t>
+  </si>
+  <si>
+    <t>BBF626</t>
+  </si>
+  <si>
+    <t>Marginal (guia platano)</t>
+  </si>
+  <si>
+    <t>dedos 3-4 (centro) algo mas amarillos</t>
+  </si>
+  <si>
+    <t>recibir con observacion y rotar primero; si va a camara, yodo</t>
+  </si>
+  <si>
+    <t>PLATANO (generico) - no comparable</t>
+  </si>
+  <si>
+    <t>en escala banana seria 4 con reserva (3-4); camara ZAC 19 (981 cajas)</t>
+  </si>
+  <si>
+    <t>11:08</t>
+  </si>
+  <si>
+    <t>#273</t>
+  </si>
+  <si>
+    <t>3/30</t>
+  </si>
+  <si>
+    <t>Fischer (via Etimex)</t>
+  </si>
+  <si>
+    <t>Daniel Ferreira Faria</t>
+  </si>
+  <si>
+    <t>IZD6D78</t>
+  </si>
+  <si>
+    <t>Marginal</t>
+  </si>
+  <si>
+    <t>medio (dedo 3)</t>
+  </si>
+  <si>
+    <t>camara corta y prioridad de despacho; cortar 5 mas de la zona del dedo 3</t>
+  </si>
+  <si>
+    <t>media (tabla blanca)</t>
+  </si>
+  <si>
+    <t>"si con la fruta en la mano se ve mas amarilla, baja a 2"</t>
+  </si>
+  <si>
+    <t>08:27</t>
+  </si>
+  <si>
+    <t>#278</t>
+  </si>
+  <si>
+    <t>BONITA</t>
+  </si>
+  <si>
+    <t>26/30</t>
+  </si>
+  <si>
+    <t>Noboa</t>
+  </si>
+  <si>
+    <t>Marco Munoz</t>
+  </si>
+  <si>
+    <t>PYCJ23</t>
+  </si>
+  <si>
+    <t>4 de 5 en 3, dedo 4 en 4</t>
+  </si>
+  <si>
+    <t>punteado pardo en el eje (dedos 1, 2, 5): ovulos, o frio subagudo (sospecha leve)</t>
+  </si>
+  <si>
+    <t>camara corta y salida rapida; si pulpa &lt; 13 C pelar dedo de frente y fondo y fotografiar cara interna</t>
+  </si>
+  <si>
+    <t>placa leida JHF560 (dudosa)</t>
+  </si>
+  <si>
+    <t>08:32</t>
+  </si>
+  <si>
+    <t>#275</t>
+  </si>
+  <si>
+    <t>PEPE</t>
+  </si>
+  <si>
+    <t>22/30</t>
+  </si>
+  <si>
+    <t>Interbanana</t>
+  </si>
+  <si>
+    <t>Daniel Alvarez</t>
+  </si>
+  <si>
+    <t>PYCJ24</t>
+  </si>
+  <si>
+    <t>Marginal (2 de 5 dedos en 2)</t>
+  </si>
+  <si>
+    <t>fondo (dedos 4-5 en 2, franja nitida, brillo humedo)</t>
+  </si>
+  <si>
+    <t>pardeo en cuello dedos 1-2 (corona); restos florales en puntas 2, 4, 5 (punta de cigarro); dedo 5 delgado, cascara gruesa</t>
+  </si>
+  <si>
+    <t>camara corta o maduracion inmediata; separar la fruta del fondo; cortar 5 mas del fondo</t>
+  </si>
+  <si>
+    <t>ticket leido "carga 05/09, descarga 28/09" (23 dias): mal leido, verificar</t>
+  </si>
+  <si>
+    <t>08:37</t>
+  </si>
+  <si>
+    <t>#279</t>
+  </si>
+  <si>
+    <t>Nobora Trading Group</t>
+  </si>
+  <si>
+    <t>Marcelo Hernandez</t>
+  </si>
+  <si>
+    <t>VHFH90</t>
+  </si>
+  <si>
+    <t>medio</t>
+  </si>
+  <si>
+    <t>ninguna (sin haces pardos, sin frio)</t>
+  </si>
+  <si>
+    <t>camara corta con prioridad de despacho; cortar 5 mas del medio</t>
+  </si>
+  <si>
+    <t>placa leida PTC-123; foto mas amarillenta y con peor luz que la 2a muestra</t>
+  </si>
+  <si>
+    <t>08:41</t>
+  </si>
+  <si>
+    <t>25/30</t>
+  </si>
+  <si>
+    <t>medio/fondo (dedos 4-5)</t>
+  </si>
+  <si>
+    <t>ninguna visible</t>
+  </si>
+  <si>
+    <t>camara corta; cortar 5 mas del fondo</t>
+  </si>
+  <si>
+    <t>segunda muestra del mismo camion</t>
+  </si>
+  <si>
+    <t>08:46</t>
+  </si>
+  <si>
+    <t>Aceptar</t>
+  </si>
+  <si>
+    <t>medio (leve)</t>
+  </si>
+  <si>
+    <t>camara segun plan; si el gradiente termico supera 4 C, cortar 5 mas del medio</t>
+  </si>
+  <si>
+    <t>mismo pallet 22/30 que la lectura de 08:37: tomar como 3-4, no dos lotes</t>
+  </si>
+  <si>
+    <t>Una fila por lectura del control por corte de Aloha (foto fija sobre la tabla del carrito, leida por IA con el protocolo UAM v1 del 16/09/2026 y confirmada por el operario). El operario dejo "3 dedos" por defecto pero en todas las fotos hay 5. La IA NO recibio temperaturas de pulpa, fecha de carga, transito ni productor (la pestana Corte no le pasa el contexto del camion). Fuente: fuentes\calidad_fotos\2026-09-25_cortes_aloha_recepcion\.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,13 +844,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -416,9 +872,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="2" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -733,29 +1191,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5043BCB7-F4A0-4C7E-BD8D-32DFFA1595AF}">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" bestFit="1" width="17.85546875" customWidth="1"/>
+    <col min="3" max="3" bestFit="1" width="9" customWidth="1"/>
+    <col min="4" max="4" bestFit="1" width="12" customWidth="1"/>
+    <col min="5" max="5" bestFit="1" width="7.5703125" customWidth="1"/>
+    <col min="6" max="6" bestFit="1" width="14" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="13.7109375" customWidth="1"/>
+    <col min="8" max="8" bestFit="1" width="11.28515625" customWidth="1"/>
+    <col min="9" max="9" bestFit="1" width="13.5703125" customWidth="1"/>
+    <col min="10" max="10" bestFit="1" width="17.28515625" customWidth="1"/>
+    <col min="11" max="11" bestFit="1" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" bestFit="1" width="13.7109375" customWidth="1"/>
+    <col min="13" max="13" bestFit="1" width="15.42578125" customWidth="1"/>
+    <col min="14" max="14" bestFit="1" width="15.5703125" customWidth="1"/>
+    <col min="15" max="15" bestFit="1" width="10" customWidth="1"/>
+    <col min="16" max="16" bestFit="1" width="13.28515625" customWidth="1"/>
+    <col min="17" max="17" bestFit="1" width="6.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -808,84 +1266,1065 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2">
+      <c r="A2" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="0">
         <v>1009</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="0">
         <v>14.5</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="0">
         <v>28.7</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="0">
         <v>24.3</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="0">
         <v>4</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="0" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3">
+      <c r="A3" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="0">
         <v>1008</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="0">
         <v>4</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="0" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4">
+      <c r="A4" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="0">
         <v>1008</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="0">
         <v>5</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="0" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46290</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="0">
+        <v>984</v>
+      </c>
+      <c r="K5" s="0">
+        <v>2</v>
+      </c>
+      <c r="O5" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q5" s="0" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46290</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="0">
+        <v>980</v>
+      </c>
+      <c r="K6" s="0">
+        <v>2</v>
+      </c>
+      <c r="O6" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q6" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46290</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="0">
+        <v>1050</v>
+      </c>
+      <c r="K7" s="0">
+        <v>2</v>
+      </c>
+      <c r="O7" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" s="0" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="2">
+        <v>46290</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="0">
+        <v>981</v>
+      </c>
+      <c r="K8" s="0">
+        <v>4</v>
+      </c>
+      <c r="O8" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q8" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="2">
+        <v>46290</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="0">
+        <v>1008</v>
+      </c>
+      <c r="K9" s="0">
+        <v>3</v>
+      </c>
+      <c r="O9" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q9" s="0" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="2">
+        <v>46291</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="0">
+        <v>1080</v>
+      </c>
+      <c r="K10" s="0">
+        <v>3</v>
+      </c>
+      <c r="O10" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q10" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="2">
+        <v>46291</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="0">
+        <v>1080</v>
+      </c>
+      <c r="K11" s="0">
+        <v>3</v>
+      </c>
+      <c r="O11" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q11" s="0" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="2">
+        <v>46291</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="0">
+        <v>1080</v>
+      </c>
+      <c r="K12" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="O12" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q12" s="0" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q1" xr:uid="{5043BCB7-F4A0-4C7E-BD8D-32DFFA1595AF}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:V13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="16" max="16" width="40" customWidth="1"/>
+    <col min="17" max="17" width="50" customWidth="1"/>
+    <col min="22" max="22" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2" s="0">
+        <v>984</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="L2" s="0">
+        <v>5</v>
+      </c>
+      <c r="M2" s="0">
+        <v>2</v>
+      </c>
+      <c r="N2" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="P2" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q2" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="R2" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T2" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U2" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V2" s="0" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="I3" s="0">
+        <v>980</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="K3" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="L3" s="0">
+        <v>5</v>
+      </c>
+      <c r="M3" s="0">
+        <v>2</v>
+      </c>
+      <c r="N3" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="O3" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="P3" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q3" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="R3" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S3" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T3" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U3" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V3" s="0" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="0">
+        <v>1050</v>
+      </c>
+      <c r="J4" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="K4" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="L4" s="0">
+        <v>5</v>
+      </c>
+      <c r="M4" s="0">
+        <v>2</v>
+      </c>
+      <c r="N4" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="O4" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="P4" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q4" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="R4" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S4" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T4" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U4" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V4" s="0" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="I5" s="0">
+        <v>981</v>
+      </c>
+      <c r="J5" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="K5" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="L5" s="0">
+        <v>5</v>
+      </c>
+      <c r="M5" s="0">
+        <v>4</v>
+      </c>
+      <c r="N5" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="O5" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="P5" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q5" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="R5" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="S5" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T5" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U5" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V5" s="0" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>46290</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="I6" s="0">
+        <v>1008</v>
+      </c>
+      <c r="J6" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="K6" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="L6" s="0">
+        <v>5</v>
+      </c>
+      <c r="M6" s="0">
+        <v>3</v>
+      </c>
+      <c r="N6" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="O6" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="P6" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q6" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="R6" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S6" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="T6" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U6" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V6" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="I7" s="0">
+        <v>1080</v>
+      </c>
+      <c r="J7" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="K7" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="L7" s="0">
+        <v>5</v>
+      </c>
+      <c r="M7" s="0">
+        <v>3</v>
+      </c>
+      <c r="N7" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="O7" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="P7" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q7" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="R7" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S7" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T7" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U7" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V7" s="0" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="I8" s="0">
+        <v>1080</v>
+      </c>
+      <c r="J8" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="K8" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="L8" s="0">
+        <v>5</v>
+      </c>
+      <c r="M8" s="0">
+        <v>3</v>
+      </c>
+      <c r="N8" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="O8" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="P8" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q8" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="R8" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S8" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T8" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U8" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V8" s="0" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="I9" s="0">
+        <v>1080</v>
+      </c>
+      <c r="J9" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="K9" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="L9" s="0">
+        <v>5</v>
+      </c>
+      <c r="M9" s="0">
+        <v>3</v>
+      </c>
+      <c r="N9" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="O9" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="P9" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q9" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="R9" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S9" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T9" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U9" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V9" s="0" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="I10" s="0">
+        <v>1080</v>
+      </c>
+      <c r="J10" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="K10" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="L10" s="0">
+        <v>5</v>
+      </c>
+      <c r="M10" s="0">
+        <v>3</v>
+      </c>
+      <c r="N10" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="O10" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="P10" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q10" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="R10" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S10" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T10" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U10" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V10" s="0" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>46291</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="I11" s="0">
+        <v>1080</v>
+      </c>
+      <c r="J11" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="K11" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="L11" s="0">
+        <v>5</v>
+      </c>
+      <c r="M11" s="0">
+        <v>4</v>
+      </c>
+      <c r="N11" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="O11" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="P11" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q11" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="R11" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="S11" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="T11" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="U11" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="V11" s="0" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>